<commit_message>
Last updates and models
</commit_message>
<xml_diff>
--- a/otros_docs/Diccionario.xlsx
+++ b/otros_docs/Diccionario.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Clases\ICESI\2024_I\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jhona\Dropbox\ASPECTOS MAESTRIA\Cursos semestres\SEMESTRE 1\ML2 - Aprendizaje automatico 2\Competencia kaggle\competencia_ml2_icesi\otros_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFF96959-91E5-442C-B911-AB8102AF9508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3195D61D-F746-4200-9035-FEEBCE12317D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="3" r:id="rId1"/>
@@ -292,7 +292,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,13 +308,56 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -329,9 +372,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -613,13 +664,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B44"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="59.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="59.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>85</v>
       </c>
@@ -627,159 +678,159 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -787,187 +838,187 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="8" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="8" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="8" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="25" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="8" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="8" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="8" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="8" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="29" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="8" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="31" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="32" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="33" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="7" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="34" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="8" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="35" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="36" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="8" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="37" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="38" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="8" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="39" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="9" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="40" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="8" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="41" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="9" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="42" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="3" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="43" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="3" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+    <row r="44" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="8" t="s">
         <v>77</v>
       </c>
     </row>

</xml_diff>